<commit_message>
update PFllamam lucia v1
spreadsheet updated
</commit_message>
<xml_diff>
--- a/PROPULSION HRD-01 Diseño de banco de pruebas Maria Rev.1.xlsx
+++ b/PROPULSION HRD-01 Diseño de banco de pruebas Maria Rev.1.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leonardo.valadez\Documents\Repositorios\rocket-benchtest-stand\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Engineering\01 Repos\rocket-benchtest-stand\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0623EDE7-AC27-4517-962E-9E622229157C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21195" windowHeight="8085" activeTab="4"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
     <sheet name="Truss design 2.0" sheetId="8" r:id="rId5"/>
     <sheet name="Instrumentation" sheetId="7" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,14 +41,14 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
   <futureMetadata name="XLRICHVALUE" count="1">
     <bk>
       <extLst>
-        <ext xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="0"/>
         </ext>
       </extLst>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="238">
   <si>
     <t>(Materials selection in mechanical design, pp 12)</t>
   </si>
@@ -852,11 +853,14 @@
   <si>
     <t>Large member</t>
   </si>
+  <si>
+    <t>Welding joint analysis</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
@@ -1230,7 +1234,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1328,6 +1332,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-DB50-479D-9043-705D97A14E93}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="6"/>
@@ -1404,6 +1413,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-DB50-479D-9043-705D97A14E93}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="7"/>
@@ -1480,6 +1494,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-DB50-479D-9043-705D97A14E93}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="8"/>
@@ -1556,6 +1575,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-DB50-479D-9043-705D97A14E93}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="9"/>
@@ -1632,6 +1656,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-DB50-479D-9043-705D97A14E93}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="0"/>
@@ -1702,6 +1731,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-DB50-479D-9043-705D97A14E93}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -1772,6 +1806,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-DB50-479D-9043-705D97A14E93}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
@@ -1842,6 +1881,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-DB50-479D-9043-705D97A14E93}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="3"/>
@@ -1912,6 +1956,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-DB50-479D-9043-705D97A14E93}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="4"/>
@@ -1982,6 +2031,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000009-DB50-479D-9043-705D97A14E93}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -2164,7 +2218,7 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -2262,6 +2316,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F9EA-4D43-95B3-60586230201B}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -2332,6 +2391,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-F9EA-4D43-95B3-60586230201B}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
@@ -2402,6 +2466,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-F9EA-4D43-95B3-60586230201B}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="3"/>
@@ -2472,6 +2541,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-F9EA-4D43-95B3-60586230201B}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -2654,7 +2728,7 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -2752,6 +2826,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="6"/>
@@ -2828,6 +2907,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="7"/>
@@ -2904,6 +2988,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="8"/>
@@ -2980,6 +3069,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="9"/>
@@ -3056,6 +3150,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="0"/>
@@ -3126,6 +3225,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -3196,6 +3300,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
@@ -3266,6 +3375,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="3"/>
@@ -3336,6 +3450,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="4"/>
@@ -3406,6 +3525,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000009-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="10"/>
@@ -3482,6 +3606,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000A-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="11"/>
@@ -3558,6 +3687,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000B-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="12"/>
@@ -3637,6 +3771,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000C-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="13"/>
@@ -3716,6 +3855,11 @@
             </c:numRef>
           </c:yVal>
           <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000D-4CAF-4C5C-9F21-EBC0F6EC3924}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -5586,7 +5730,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5684C3C5-DAA1-0FFD-42E3-3D5DF59271BC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5684C3C5-DAA1-0FFD-42E3-3D5DF59271BC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5635,7 +5779,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{896B3375-9C92-1B6B-758A-EA72BB08F586}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{896B3375-9C92-1B6B-758A-EA72BB08F586}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5679,7 +5823,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6CA22387-73AB-26F5-3C1D-5737F039543F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6CA22387-73AB-26F5-3C1D-5737F039543F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5728,7 +5872,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D8E8793-F09C-DBBC-8F68-AB2AB1330A6F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D8E8793-F09C-DBBC-8F68-AB2AB1330A6F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5772,7 +5916,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED8B252A-7486-70B0-AC76-61C6891FB4D2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED8B252A-7486-70B0-AC76-61C6891FB4D2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5821,7 +5965,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7C4DA1F8-A635-4E4C-9C97-10B5703E0C0F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7C4DA1F8-A635-4E4C-9C97-10B5703E0C0F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5882,7 +6026,7 @@
         <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{401281D1-570F-B0E7-290B-B831A7033209}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{401281D1-570F-B0E7-290B-B831A7033209}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5945,7 +6089,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -5975,7 +6125,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -6005,7 +6161,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3"/>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
@@ -6045,7 +6207,7 @@
         <xdr:cNvPr id="6145" name="AutoShape 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2CF56B6D-0E4C-76D3-7C78-C253C736FF53}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2CF56B6D-0E4C-76D3-7C78-C253C736FF53}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6458,16 +6620,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:R27"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="2:18" ht="15" thickBot="1">
       <c r="I2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:18" ht="15.75" thickBot="1">
+    <row r="3" spans="2:18" ht="15" thickBot="1">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -6539,7 +6701,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="2:18" ht="15">
+    <row r="12" spans="2:18">
       <c r="B12" t="s">
         <v>19</v>
       </c>
@@ -6630,7 +6792,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R6" r:id="rId1"/>
+    <hyperlink ref="R6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
@@ -6639,18 +6801,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:N121"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="8.875" style="4"/>
-    <col min="2" max="2" width="18.875" style="4" customWidth="1"/>
-    <col min="3" max="10" width="8.875" style="4"/>
+    <col min="1" max="1" width="8.90625" style="4"/>
+    <col min="2" max="2" width="18.90625" style="4" customWidth="1"/>
+    <col min="3" max="10" width="8.90625" style="4"/>
     <col min="11" max="11" width="18" style="4" customWidth="1"/>
-    <col min="12" max="12" width="23.25" style="4" customWidth="1"/>
-    <col min="13" max="13" width="8.875" style="4"/>
-    <col min="14" max="14" width="30.875" style="4" customWidth="1"/>
-    <col min="15" max="16384" width="8.875" style="4"/>
+    <col min="12" max="12" width="23.26953125" style="4" customWidth="1"/>
+    <col min="13" max="13" width="8.90625" style="4"/>
+    <col min="14" max="14" width="30.90625" style="4" customWidth="1"/>
+    <col min="15" max="16384" width="8.90625" style="4"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:14" ht="15" thickBot="1"/>
@@ -6716,7 +6878,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="2:14" ht="15.75" thickBot="1">
+    <row r="5" spans="2:14" ht="15" thickBot="1">
       <c r="B5" s="10"/>
       <c r="C5" s="11">
         <v>18</v>
@@ -6737,7 +6899,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="2:14" ht="15">
+    <row r="6" spans="2:14">
       <c r="B6" s="6" t="s">
         <v>52</v>
       </c>
@@ -6766,7 +6928,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="2:14" ht="15.75" thickBot="1">
+    <row r="7" spans="2:14" ht="15" thickBot="1">
       <c r="B7" s="10"/>
       <c r="C7" s="11">
         <v>18</v>
@@ -6787,7 +6949,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="2:14" ht="15">
+    <row r="8" spans="2:14">
       <c r="B8" s="6" t="s">
         <v>55</v>
       </c>
@@ -6810,7 +6972,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="2:14" ht="15">
+    <row r="9" spans="2:14">
       <c r="B9" s="13"/>
       <c r="C9" s="11">
         <v>18</v>
@@ -6831,7 +6993,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="2:14" ht="15">
+    <row r="10" spans="2:14">
       <c r="B10" s="13"/>
       <c r="C10" s="11">
         <v>16</v>
@@ -6852,7 +7014,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="2:14" ht="15.75" thickBot="1">
+    <row r="11" spans="2:14" ht="15" thickBot="1">
       <c r="B11" s="10"/>
       <c r="C11" s="11">
         <v>14</v>
@@ -6873,7 +7035,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="2:14" ht="15">
+    <row r="12" spans="2:14">
       <c r="B12" s="6" t="s">
         <v>56</v>
       </c>
@@ -6896,7 +7058,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="2:14" ht="15">
+    <row r="13" spans="2:14">
       <c r="B13" s="13"/>
       <c r="C13" s="11">
         <v>18</v>
@@ -6917,7 +7079,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="2:14" ht="15">
+    <row r="14" spans="2:14">
       <c r="B14" s="13"/>
       <c r="C14" s="11">
         <v>16</v>
@@ -6938,7 +7100,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="2:14" ht="15">
+    <row r="15" spans="2:14">
       <c r="B15" s="13"/>
       <c r="C15" s="11">
         <v>14</v>
@@ -6959,7 +7121,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="2:14" ht="15">
+    <row r="16" spans="2:14">
       <c r="B16" s="13"/>
       <c r="C16" s="11">
         <v>13</v>
@@ -6980,7 +7142,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="2:8" ht="15">
+    <row r="17" spans="2:8">
       <c r="B17" s="13"/>
       <c r="C17" s="11">
         <v>12</v>
@@ -7001,7 +7163,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="15">
+    <row r="18" spans="2:8">
       <c r="B18" s="13"/>
       <c r="C18" s="11">
         <v>11</v>
@@ -7022,7 +7184,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="15.75" thickBot="1">
+    <row r="19" spans="2:8" ht="15" thickBot="1">
       <c r="B19" s="10"/>
       <c r="C19" s="11">
         <v>10</v>
@@ -7043,7 +7205,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="2:8" ht="15">
+    <row r="20" spans="2:8">
       <c r="B20" s="6" t="s">
         <v>58</v>
       </c>
@@ -7066,7 +7228,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="2:8" ht="15">
+    <row r="21" spans="2:8">
       <c r="B21" s="13"/>
       <c r="C21" s="11">
         <v>18</v>
@@ -7087,7 +7249,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="2:8" ht="15">
+    <row r="22" spans="2:8">
       <c r="B22" s="13"/>
       <c r="C22" s="11">
         <v>16</v>
@@ -7108,7 +7270,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="2:8" ht="15">
+    <row r="23" spans="2:8">
       <c r="B23" s="13"/>
       <c r="C23" s="11">
         <v>14</v>
@@ -7129,7 +7291,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="2:8" ht="15.75" thickBot="1">
+    <row r="24" spans="2:8" ht="15" thickBot="1">
       <c r="B24" s="10"/>
       <c r="C24" s="11">
         <v>12</v>
@@ -7150,7 +7312,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="2:8" ht="15">
+    <row r="25" spans="2:8">
       <c r="B25" s="6" t="s">
         <v>59</v>
       </c>
@@ -7173,7 +7335,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="2:8" ht="15">
+    <row r="26" spans="2:8">
       <c r="B26" s="13"/>
       <c r="C26" s="11">
         <v>18</v>
@@ -7194,7 +7356,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="2:8" ht="15">
+    <row r="27" spans="2:8">
       <c r="B27" s="13"/>
       <c r="C27" s="11">
         <v>16</v>
@@ -7215,7 +7377,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="2:8" ht="15">
+    <row r="28" spans="2:8">
       <c r="B28" s="13"/>
       <c r="C28" s="11">
         <v>14</v>
@@ -7236,7 +7398,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="29" spans="2:8" ht="15">
+    <row r="29" spans="2:8">
       <c r="B29" s="13"/>
       <c r="C29" s="11">
         <v>12</v>
@@ -7257,7 +7419,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="2:8" ht="15.75" thickBot="1">
+    <row r="30" spans="2:8" ht="15" thickBot="1">
       <c r="B30" s="10"/>
       <c r="C30" s="11">
         <v>9</v>
@@ -7278,7 +7440,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="2:8" ht="15">
+    <row r="31" spans="2:8">
       <c r="B31" s="6" t="s">
         <v>60</v>
       </c>
@@ -7301,7 +7463,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="2:8" ht="15">
+    <row r="32" spans="2:8">
       <c r="B32" s="13"/>
       <c r="C32" s="11">
         <v>14</v>
@@ -7322,7 +7484,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="2:9" ht="15">
+    <row r="33" spans="2:9">
       <c r="B33" s="13"/>
       <c r="C33" s="11">
         <v>12</v>
@@ -7343,7 +7505,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="2:9" ht="15">
+    <row r="34" spans="2:9">
       <c r="B34" s="13"/>
       <c r="C34" s="11">
         <v>10</v>
@@ -7364,7 +7526,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="35" spans="2:9" ht="15.75" thickBot="1">
+    <row r="35" spans="2:9" ht="15" thickBot="1">
       <c r="B35" s="10"/>
       <c r="C35" s="11">
         <v>9</v>
@@ -7385,7 +7547,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="2:9" ht="15">
+    <row r="36" spans="2:9">
       <c r="B36" s="6" t="s">
         <v>61</v>
       </c>
@@ -7408,7 +7570,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="37" spans="2:9" ht="15">
+    <row r="37" spans="2:9">
       <c r="B37" s="13"/>
       <c r="C37" s="11">
         <v>11</v>
@@ -7429,7 +7591,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="2:9" ht="15">
+    <row r="38" spans="2:9">
       <c r="B38" s="13"/>
       <c r="C38" s="11">
         <v>7</v>
@@ -7450,7 +7612,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="39" spans="2:9" ht="15.75" thickBot="1">
+    <row r="39" spans="2:9" ht="15" thickBot="1">
       <c r="B39" s="10"/>
       <c r="C39" s="11" t="s">
         <v>62</v>
@@ -7471,7 +7633,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="40" spans="2:9" ht="15">
+    <row r="40" spans="2:9">
       <c r="B40" s="6" t="s">
         <v>63</v>
       </c>
@@ -7494,7 +7656,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="41" spans="2:9" ht="28.5">
+    <row r="41" spans="2:9" ht="29">
       <c r="B41" s="13"/>
       <c r="C41" s="11">
         <v>11</v>
@@ -7515,7 +7677,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="42" spans="2:9" ht="15">
+    <row r="42" spans="2:9">
       <c r="B42" s="13"/>
       <c r="C42" s="11">
         <v>9</v>
@@ -7536,7 +7698,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="2:9" ht="15">
+    <row r="43" spans="2:9">
       <c r="B43" s="13"/>
       <c r="C43" s="11">
         <v>7</v>
@@ -7557,7 +7719,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="44" spans="2:9" ht="29.25" thickBot="1">
+    <row r="44" spans="2:9" ht="29.5" thickBot="1">
       <c r="B44" s="10"/>
       <c r="C44" s="11" t="s">
         <v>62</v>
@@ -7578,7 +7740,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="45" spans="2:9" ht="15">
+    <row r="45" spans="2:9">
       <c r="B45" s="6" t="s">
         <v>65</v>
       </c>
@@ -7601,7 +7763,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="46" spans="2:9" ht="15.75" thickBot="1">
+    <row r="46" spans="2:9" ht="15" thickBot="1">
       <c r="B46" s="13"/>
       <c r="C46" s="11">
         <v>9</v>
@@ -7622,7 +7784,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="47" spans="2:9" ht="15.75" thickBot="1">
+    <row r="47" spans="2:9" ht="15" thickBot="1">
       <c r="B47" s="13"/>
       <c r="C47" s="11">
         <v>7</v>
@@ -7644,7 +7806,7 @@
       </c>
       <c r="I47" s="1"/>
     </row>
-    <row r="48" spans="2:9" ht="29.25" thickBot="1">
+    <row r="48" spans="2:9" ht="29.5" thickBot="1">
       <c r="B48" s="10"/>
       <c r="C48" s="11" t="s">
         <v>62</v>
@@ -7665,7 +7827,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="49" spans="2:9" ht="15">
+    <row r="49" spans="2:9">
       <c r="B49" s="6" t="s">
         <v>67</v>
       </c>
@@ -7688,7 +7850,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="2:9" ht="29.25" thickBot="1">
+    <row r="50" spans="2:9" ht="29.5" thickBot="1">
       <c r="B50" s="13"/>
       <c r="C50" s="11" t="s">
         <v>68</v>
@@ -7709,7 +7871,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="51" spans="2:9" ht="15.75" thickBot="1">
+    <row r="51" spans="2:9" ht="15" thickBot="1">
       <c r="B51" s="13"/>
       <c r="C51" s="11">
         <v>9</v>
@@ -7731,7 +7893,7 @@
       </c>
       <c r="I51" s="1"/>
     </row>
-    <row r="52" spans="2:9" ht="28.5">
+    <row r="52" spans="2:9" ht="29">
       <c r="B52" s="13"/>
       <c r="C52" s="11" t="s">
         <v>69</v>
@@ -7752,7 +7914,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="53" spans="2:9" ht="29.25" thickBot="1">
+    <row r="53" spans="2:9" ht="29.5" thickBot="1">
       <c r="B53" s="10"/>
       <c r="C53" s="11" t="s">
         <v>62</v>
@@ -7773,7 +7935,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="54" spans="2:9" ht="28.5">
+    <row r="54" spans="2:9" ht="29">
       <c r="B54" s="6" t="s">
         <v>70</v>
       </c>
@@ -7796,7 +7958,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="55" spans="2:9" ht="28.5">
+    <row r="55" spans="2:9" ht="29">
       <c r="B55" s="13"/>
       <c r="C55" s="11" t="s">
         <v>69</v>
@@ -7817,7 +7979,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="56" spans="2:9" ht="29.25" thickBot="1">
+    <row r="56" spans="2:9" ht="29.5" thickBot="1">
       <c r="B56" s="10"/>
       <c r="C56" s="14" t="s">
         <v>62</v>
@@ -7862,7 +8024,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="60" spans="2:9" ht="15.75" thickBot="1">
+    <row r="60" spans="2:9" ht="15" thickBot="1">
       <c r="B60" s="10" t="s">
         <v>72</v>
       </c>
@@ -7885,7 +8047,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="61" spans="2:9" ht="15">
+    <row r="61" spans="2:9">
       <c r="B61" s="6" t="s">
         <v>73</v>
       </c>
@@ -7908,7 +8070,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="62" spans="2:9" ht="15.75" thickBot="1">
+    <row r="62" spans="2:9" ht="15" thickBot="1">
       <c r="B62" s="10"/>
       <c r="C62" s="11">
         <v>18</v>
@@ -7929,7 +8091,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="63" spans="2:9" ht="15">
+    <row r="63" spans="2:9">
       <c r="B63" s="6" t="s">
         <v>74</v>
       </c>
@@ -7952,7 +8114,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="64" spans="2:9" ht="15.75" thickBot="1">
+    <row r="64" spans="2:9" ht="15" thickBot="1">
       <c r="B64" s="10"/>
       <c r="C64" s="11">
         <v>18</v>
@@ -7973,7 +8135,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="65" spans="2:8" ht="15">
+    <row r="65" spans="2:8">
       <c r="B65" s="6" t="s">
         <v>75</v>
       </c>
@@ -7996,7 +8158,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="66" spans="2:8" ht="15">
+    <row r="66" spans="2:8">
       <c r="B66" s="13"/>
       <c r="C66" s="11">
         <v>18</v>
@@ -8017,7 +8179,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="67" spans="2:8" ht="15">
+    <row r="67" spans="2:8">
       <c r="B67" s="13"/>
       <c r="C67" s="11">
         <v>16</v>
@@ -8038,7 +8200,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="68" spans="2:8" ht="15">
+    <row r="68" spans="2:8">
       <c r="B68" s="13"/>
       <c r="C68" s="11">
         <v>14</v>
@@ -8059,7 +8221,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="69" spans="2:8" ht="15.75" thickBot="1">
+    <row r="69" spans="2:8" ht="15" thickBot="1">
       <c r="B69" s="10"/>
       <c r="C69" s="11">
         <v>11</v>
@@ -8080,7 +8242,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="70" spans="2:8" ht="15">
+    <row r="70" spans="2:8">
       <c r="B70" s="6" t="s">
         <v>76</v>
       </c>
@@ -8103,7 +8265,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="71" spans="2:8" ht="15.75" thickBot="1">
+    <row r="71" spans="2:8" ht="15" thickBot="1">
       <c r="B71" s="10"/>
       <c r="C71" s="11">
         <v>18</v>
@@ -8124,7 +8286,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="72" spans="2:8" ht="15">
+    <row r="72" spans="2:8">
       <c r="B72" s="6" t="s">
         <v>77</v>
       </c>
@@ -8147,7 +8309,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="73" spans="2:8" ht="15">
+    <row r="73" spans="2:8">
       <c r="B73" s="13"/>
       <c r="C73" s="11">
         <v>18</v>
@@ -8168,7 +8330,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="74" spans="2:8" ht="15">
+    <row r="74" spans="2:8">
       <c r="B74" s="13"/>
       <c r="C74" s="11">
         <v>14</v>
@@ -8189,7 +8351,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="75" spans="2:8" ht="15.75" thickBot="1">
+    <row r="75" spans="2:8" ht="15" thickBot="1">
       <c r="B75" s="10"/>
       <c r="C75" s="11">
         <v>11</v>
@@ -8210,7 +8372,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="76" spans="2:8" ht="15">
+    <row r="76" spans="2:8">
       <c r="B76" s="6" t="s">
         <v>78</v>
       </c>
@@ -8233,7 +8395,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="77" spans="2:8" ht="15.75" thickBot="1">
+    <row r="77" spans="2:8" ht="15" thickBot="1">
       <c r="B77" s="10"/>
       <c r="C77" s="11">
         <v>18</v>
@@ -8254,7 +8416,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="78" spans="2:8" ht="15">
+    <row r="78" spans="2:8">
       <c r="B78" s="6" t="s">
         <v>79</v>
       </c>
@@ -8277,7 +8439,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="79" spans="2:8" ht="15">
+    <row r="79" spans="2:8">
       <c r="B79" s="13"/>
       <c r="C79" s="11">
         <v>18</v>
@@ -8298,7 +8460,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="80" spans="2:8" ht="15.75" thickBot="1">
+    <row r="80" spans="2:8" ht="15" thickBot="1">
       <c r="B80" s="10"/>
       <c r="C80" s="11">
         <v>14</v>
@@ -8319,7 +8481,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="81" spans="2:8" ht="15.75" thickBot="1">
+    <row r="81" spans="2:8" ht="15" thickBot="1">
       <c r="B81" s="17" t="s">
         <v>81</v>
       </c>
@@ -8342,7 +8504,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="82" spans="2:8" ht="15">
+    <row r="82" spans="2:8">
       <c r="B82" s="6" t="s">
         <v>82</v>
       </c>
@@ -8365,7 +8527,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="83" spans="2:8" ht="15">
+    <row r="83" spans="2:8">
       <c r="B83" s="13"/>
       <c r="C83" s="11">
         <v>16</v>
@@ -8386,7 +8548,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="84" spans="2:8" ht="15">
+    <row r="84" spans="2:8">
       <c r="B84" s="13"/>
       <c r="C84" s="11">
         <v>14</v>
@@ -8407,7 +8569,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="85" spans="2:8" ht="15">
+    <row r="85" spans="2:8">
       <c r="B85" s="13"/>
       <c r="C85" s="11">
         <v>11</v>
@@ -8428,7 +8590,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="86" spans="2:8" ht="15.75" thickBot="1">
+    <row r="86" spans="2:8" ht="15" thickBot="1">
       <c r="B86" s="10"/>
       <c r="C86" s="11">
         <v>10</v>
@@ -8446,7 +8608,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="87" spans="2:8" ht="15">
+    <row r="87" spans="2:8">
       <c r="B87" s="6" t="s">
         <v>83</v>
       </c>
@@ -8469,7 +8631,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="88" spans="2:8" ht="15">
+    <row r="88" spans="2:8">
       <c r="B88" s="13"/>
       <c r="C88" s="11">
         <v>18</v>
@@ -8490,7 +8652,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="89" spans="2:8" ht="15">
+    <row r="89" spans="2:8">
       <c r="B89" s="13"/>
       <c r="C89" s="11">
         <v>14</v>
@@ -8511,7 +8673,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="90" spans="2:8" ht="15.75" thickBot="1">
+    <row r="90" spans="2:8" ht="15" thickBot="1">
       <c r="B90" s="10"/>
       <c r="C90" s="11">
         <v>11</v>
@@ -8532,7 +8694,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="91" spans="2:8" ht="15">
+    <row r="91" spans="2:8">
       <c r="B91" s="6" t="s">
         <v>84</v>
       </c>
@@ -8555,7 +8717,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="92" spans="2:8" ht="15">
+    <row r="92" spans="2:8">
       <c r="B92" s="13"/>
       <c r="C92" s="11">
         <v>11</v>
@@ -8576,7 +8738,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="93" spans="2:8" ht="15">
+    <row r="93" spans="2:8">
       <c r="B93" s="13"/>
       <c r="C93" s="11">
         <v>10</v>
@@ -8597,7 +8759,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="94" spans="2:8" ht="15">
+    <row r="94" spans="2:8">
       <c r="B94" s="13"/>
       <c r="C94" s="11">
         <v>7</v>
@@ -8618,7 +8780,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="95" spans="2:8" ht="15.75" thickBot="1">
+    <row r="95" spans="2:8" ht="15" thickBot="1">
       <c r="B95" s="10"/>
       <c r="C95" s="11" t="s">
         <v>62</v>
@@ -8639,7 +8801,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="96" spans="2:8" ht="15.75" thickBot="1">
+    <row r="96" spans="2:8" ht="15" thickBot="1">
       <c r="B96" s="17" t="s">
         <v>85</v>
       </c>
@@ -8662,7 +8824,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="97" spans="2:8" ht="15">
+    <row r="97" spans="2:8">
       <c r="B97" s="6" t="s">
         <v>86</v>
       </c>
@@ -8685,7 +8847,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="98" spans="2:8" ht="15">
+    <row r="98" spans="2:8">
       <c r="B98" s="13"/>
       <c r="C98" s="11">
         <v>11</v>
@@ -8706,7 +8868,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="99" spans="2:8" ht="15">
+    <row r="99" spans="2:8">
       <c r="B99" s="13"/>
       <c r="C99" s="11">
         <v>9</v>
@@ -8727,7 +8889,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="100" spans="2:8" ht="15">
+    <row r="100" spans="2:8">
       <c r="B100" s="13"/>
       <c r="C100" s="11">
         <v>7</v>
@@ -8748,7 +8910,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="101" spans="2:8" ht="29.25" thickBot="1">
+    <row r="101" spans="2:8" ht="29.5" thickBot="1">
       <c r="B101" s="10"/>
       <c r="C101" s="11" t="s">
         <v>62</v>
@@ -8769,7 +8931,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="102" spans="2:8" ht="15">
+    <row r="102" spans="2:8">
       <c r="B102" s="6" t="s">
         <v>87</v>
       </c>
@@ -8792,7 +8954,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="103" spans="2:8" ht="15">
+    <row r="103" spans="2:8">
       <c r="B103" s="13"/>
       <c r="C103" s="11">
         <v>11</v>
@@ -8813,7 +8975,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="104" spans="2:8" ht="28.5">
+    <row r="104" spans="2:8" ht="29">
       <c r="B104" s="13"/>
       <c r="C104" s="11">
         <v>9</v>
@@ -8834,7 +8996,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="105" spans="2:8" ht="15">
+    <row r="105" spans="2:8">
       <c r="B105" s="13"/>
       <c r="C105" s="11">
         <v>7</v>
@@ -8855,7 +9017,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="106" spans="2:8" ht="29.25" thickBot="1">
+    <row r="106" spans="2:8" ht="29.5" thickBot="1">
       <c r="B106" s="10"/>
       <c r="C106" s="11" t="s">
         <v>62</v>
@@ -8876,7 +9038,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="107" spans="2:8" ht="15">
+    <row r="107" spans="2:8">
       <c r="B107" s="6" t="s">
         <v>88</v>
       </c>
@@ -8899,7 +9061,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="108" spans="2:8" ht="15.75" thickBot="1">
+    <row r="108" spans="2:8" ht="15" thickBot="1">
       <c r="B108" s="10"/>
       <c r="C108" s="11">
         <v>7</v>
@@ -8920,7 +9082,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="109" spans="2:8" ht="15">
+    <row r="109" spans="2:8">
       <c r="B109" s="6" t="s">
         <v>89</v>
       </c>
@@ -8943,7 +9105,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="110" spans="2:8" ht="28.5">
+    <row r="110" spans="2:8" ht="29">
       <c r="B110" s="13"/>
       <c r="C110" s="11" t="s">
         <v>68</v>
@@ -8964,7 +9126,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="111" spans="2:8" ht="28.5">
+    <row r="111" spans="2:8" ht="29">
       <c r="B111" s="13"/>
       <c r="C111" s="11" t="s">
         <v>69</v>
@@ -8985,7 +9147,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="112" spans="2:8" ht="29.25" thickBot="1">
+    <row r="112" spans="2:8" ht="29.5" thickBot="1">
       <c r="B112" s="10"/>
       <c r="C112" s="11" t="s">
         <v>62</v>
@@ -9006,7 +9168,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="113" spans="2:8" ht="15">
+    <row r="113" spans="2:8">
       <c r="B113" s="6" t="s">
         <v>90</v>
       </c>
@@ -9029,7 +9191,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="114" spans="2:8" ht="28.5">
+    <row r="114" spans="2:8" ht="29">
       <c r="B114" s="13"/>
       <c r="C114" s="11" t="s">
         <v>68</v>
@@ -9050,7 +9212,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="115" spans="2:8" ht="28.5">
+    <row r="115" spans="2:8" ht="29">
       <c r="B115" s="13"/>
       <c r="C115" s="11" t="s">
         <v>69</v>
@@ -9071,7 +9233,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="116" spans="2:8" ht="29.25" thickBot="1">
+    <row r="116" spans="2:8" ht="29.5" thickBot="1">
       <c r="B116" s="10"/>
       <c r="C116" s="11" t="s">
         <v>62</v>
@@ -9092,7 +9254,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="117" spans="2:8" ht="28.5">
+    <row r="117" spans="2:8" ht="29">
       <c r="B117" s="6" t="s">
         <v>91</v>
       </c>
@@ -9115,7 +9277,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="118" spans="2:8" ht="28.5">
+    <row r="118" spans="2:8" ht="29">
       <c r="B118" s="13"/>
       <c r="C118" s="11" t="s">
         <v>69</v>
@@ -9136,7 +9298,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="119" spans="2:8" ht="29.25" thickBot="1">
+    <row r="119" spans="2:8" ht="29.5" thickBot="1">
       <c r="B119" s="10"/>
       <c r="C119" s="11" t="s">
         <v>62</v>
@@ -9157,7 +9319,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="120" spans="2:8" ht="15">
+    <row r="120" spans="2:8">
       <c r="B120" s="6" t="s">
         <v>92</v>
       </c>
@@ -9180,7 +9342,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="121" spans="2:8" ht="15.75" thickBot="1">
+    <row r="121" spans="2:8" ht="15" thickBot="1">
       <c r="B121" s="10"/>
       <c r="C121" s="14" t="s">
         <v>69</v>
@@ -9206,9 +9368,9 @@
     <mergeCell ref="K3:L3"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="L4" r:id="rId1"/>
-    <hyperlink ref="N4" r:id="rId2" display="https://www.nan-steel.com/news/astm-a500-grade-b.html"/>
-    <hyperlink ref="L6" r:id="rId3" display="https://www.fortacero.com/cat_ptr/"/>
+    <hyperlink ref="L4" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="N4" r:id="rId2" display="https://www.nan-steel.com/news/astm-a500-grade-b.html" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="L6" r:id="rId3" display="https://www.fortacero.com/cat_ptr/" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId4"/>
@@ -9216,9 +9378,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B24:J75"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="B24:J79"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="24" spans="2:10">
       <c r="B24" t="s">
@@ -9543,6 +9705,12 @@
     <row r="75" spans="2:3">
       <c r="B75" t="s">
         <v>164</v>
+      </c>
+    </row>
+    <row r="77" spans="2:3" s="23" customFormat="1" ht="4" customHeight="1"/>
+    <row r="79" spans="2:3">
+      <c r="B79" t="s">
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -9552,9 +9720,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:W36"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="13:19">
       <c r="M2" t="s">
@@ -9786,11 +9954,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B1:F38"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="16.125" customWidth="1"/>
+    <col min="2" max="2" width="16.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="15" thickBot="1"/>
@@ -9903,7 +10071,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="14" spans="2:6" ht="28.5">
+    <row r="14" spans="2:6" ht="29">
       <c r="B14" s="24" t="s">
         <v>234</v>
       </c>
@@ -10224,9 +10392,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B3:J231"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="3" spans="2:10">
       <c r="B3" t="s">
@@ -12268,10 +12436,10 @@
     <mergeCell ref="B6:H226"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1" display="https://es.aliexpress.com/item/1005006070642588.html?spm=a2g0o.detail.1000023.7.6731h1Sth1St9k&amp;gatewayAdapt=glo2esp"/>
-    <hyperlink ref="J7" r:id="rId2" display="https://es.aliexpress.com/item/1005006236153559.html?spm=a2g0o.detail.pcDetailTopMoreOtherSeller.10.42b5Hp0XHp0XEL&amp;gps-id=pcDetailTopMoreOtherSeller&amp;scm=1007.40000.327270.0&amp;scm_id=1007.40000.327270.0&amp;scm-url=1007.40000.327270.0&amp;pvid=8e8df423-9348-430e-bd8a-ef2b74523ad3&amp;_t=gps-id:pcDetailTopMoreOtherSeller,scm-url:1007.40000.327270.0,pvid:8e8df423-9348-430e-bd8a-ef2b74523ad3,tpp_buckets:668%232846%238115%232000&amp;pdp_npi=4%40dis%21MXN%211440.14%211440.14%21%21%21580.00%21580.00%21%402101c80217210782867234885e2967%2112000036407770943%21rec%21MX%21%21AB&amp;utparam-url=scene%3ApcDetailTopMoreOtherSeller%7Cquery_from%3A&amp;search_p4p_id=202407151418067686820644873943000265_9"/>
-    <hyperlink ref="J9" r:id="rId3" display="https://es.aliexpress.com/item/1005006732452379.html?spm=a2g0o.detail.pcDetailBottomMoreOtherSeller.7.1a3d4wrx4wrxGR&amp;gps-id=pcDetailBottomMoreOtherSeller&amp;scm=1007.40000.326746.0&amp;scm_id=1007.40000.326746.0&amp;scm-url=1007.40000.326746.0&amp;pvid=b897bdac-172d-4dcc-83a0-454806878ae4&amp;_t=gps-id:pcDetailBottomMoreOtherSeller,scm-url:1007.40000.326746.0,pvid:b897bdac-172d-4dcc-83a0-454806878ae4,tpp_buckets:668%232846%238115%23870&amp;pdp_npi=4%40dis%21MXN%211253.72%21674.56%21%21%21504.92%21271.67%21%402101dee017210836143727304e969f%2112000038120783793%21rec%21MX%21%21AB&amp;utparam-url=scene%3ApcDetailBottomMoreOtherSeller%7Cquery_from%3A"/>
-    <hyperlink ref="B231" r:id="rId4" display="https://www.amazon.com.mx/Conversi%C3%B3n-Anal%C3%B3gico-Adquisici%C3%B3n-Precisi%C3%B3n-Anal%C3%B3gicas/dp/B099KR3ZH2/ref=sr_1_4_sspa?__mk_es_MX=%C3%85M%C3%85%C5%BD%C3%95%C3%91&amp;crid=2ZSLGVRH28XV4&amp;dib=eyJ2IjoiMSJ9.4G6WaOCAu0novMMLXdnrGg.WiLun_ccVPpdns00fxZXsuGMPfwrG2LR9eMn6e7xYY4&amp;dib_tag=se&amp;keywords=adc+high+sps&amp;qid=1739164832&amp;sprefix=adc+high+sps%2Caps%2C118&amp;sr=8-4-spons&amp;ufe=app_do%3Aamzn1.fos.45030d3a-91a9-4303-890a-776dee9077c1&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9tdGY&amp;psc=1"/>
+    <hyperlink ref="B4" r:id="rId1" display="https://es.aliexpress.com/item/1005006070642588.html?spm=a2g0o.detail.1000023.7.6731h1Sth1St9k&amp;gatewayAdapt=glo2esp" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
+    <hyperlink ref="J7" r:id="rId2" display="https://es.aliexpress.com/item/1005006236153559.html?spm=a2g0o.detail.pcDetailTopMoreOtherSeller.10.42b5Hp0XHp0XEL&amp;gps-id=pcDetailTopMoreOtherSeller&amp;scm=1007.40000.327270.0&amp;scm_id=1007.40000.327270.0&amp;scm-url=1007.40000.327270.0&amp;pvid=8e8df423-9348-430e-bd8a-ef2b74523ad3&amp;_t=gps-id:pcDetailTopMoreOtherSeller,scm-url:1007.40000.327270.0,pvid:8e8df423-9348-430e-bd8a-ef2b74523ad3,tpp_buckets:668%232846%238115%232000&amp;pdp_npi=4%40dis%21MXN%211440.14%211440.14%21%21%21580.00%21580.00%21%402101c80217210782867234885e2967%2112000036407770943%21rec%21MX%21%21AB&amp;utparam-url=scene%3ApcDetailTopMoreOtherSeller%7Cquery_from%3A&amp;search_p4p_id=202407151418067686820644873943000265_9" xr:uid="{00000000-0004-0000-0500-000001000000}"/>
+    <hyperlink ref="J9" r:id="rId3" display="https://es.aliexpress.com/item/1005006732452379.html?spm=a2g0o.detail.pcDetailBottomMoreOtherSeller.7.1a3d4wrx4wrxGR&amp;gps-id=pcDetailBottomMoreOtherSeller&amp;scm=1007.40000.326746.0&amp;scm_id=1007.40000.326746.0&amp;scm-url=1007.40000.326746.0&amp;pvid=b897bdac-172d-4dcc-83a0-454806878ae4&amp;_t=gps-id:pcDetailBottomMoreOtherSeller,scm-url:1007.40000.326746.0,pvid:b897bdac-172d-4dcc-83a0-454806878ae4,tpp_buckets:668%232846%238115%23870&amp;pdp_npi=4%40dis%21MXN%211253.72%21674.56%21%21%21504.92%21271.67%21%402101dee017210836143727304e969f%2112000038120783793%21rec%21MX%21%21AB&amp;utparam-url=scene%3ApcDetailBottomMoreOtherSeller%7Cquery_from%3A" xr:uid="{00000000-0004-0000-0500-000002000000}"/>
+    <hyperlink ref="B231" r:id="rId4" display="https://www.amazon.com.mx/Conversi%C3%B3n-Anal%C3%B3gico-Adquisici%C3%B3n-Precisi%C3%B3n-Anal%C3%B3gicas/dp/B099KR3ZH2/ref=sr_1_4_sspa?__mk_es_MX=%C3%85M%C3%85%C5%BD%C3%95%C3%91&amp;crid=2ZSLGVRH28XV4&amp;dib=eyJ2IjoiMSJ9.4G6WaOCAu0novMMLXdnrGg.WiLun_ccVPpdns00fxZXsuGMPfwrG2LR9eMn6e7xYY4&amp;dib_tag=se&amp;keywords=adc+high+sps&amp;qid=1739164832&amp;sprefix=adc+high+sps%2Caps%2C118&amp;sr=8-4-spons&amp;ufe=app_do%3Aamzn1.fos.45030d3a-91a9-4303-890a-776dee9077c1&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9tdGY&amp;psc=1" xr:uid="{00000000-0004-0000-0500-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId5"/>
@@ -12279,26 +12447,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d7929c02-2ff7-4e2f-b3f4-5d7437463a37" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f5cf7016-d570-4e66-bed5-9c66354e4d60">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006416C8A108E61840AFB84A4598B73E55" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b1d8d0092a91b491fa162699921cd7b6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f5cf7016-d570-4e66-bed5-9c66354e4d60" xmlns:ns3="d7929c02-2ff7-4e2f-b3f4-5d7437463a37" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dc769dae83c42ca581dc5110a4ef7ce3" ns2:_="" ns3:_="">
     <xsd:import namespace="f5cf7016-d570-4e66-bed5-9c66354e4d60"/>
@@ -12505,26 +12653,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B672EAD0-EA6C-460E-95E6-5BDD1102E907}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d7929c02-2ff7-4e2f-b3f4-5d7437463a37"/>
-    <ds:schemaRef ds:uri="f5cf7016-d570-4e66-bed5-9c66354e4d60"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2573117B-6260-4644-A359-931F1507CA1F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d7929c02-2ff7-4e2f-b3f4-5d7437463a37" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f5cf7016-d570-4e66-bed5-9c66354e4d60">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11299929-15DA-49D6-A514-2A8A25D7CF50}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12541,4 +12690,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2573117B-6260-4644-A359-931F1507CA1F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B672EAD0-EA6C-460E-95E6-5BDD1102E907}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d7929c02-2ff7-4e2f-b3f4-5d7437463a37"/>
+    <ds:schemaRef ds:uri="f5cf7016-d570-4e66-bed5-9c66354e4d60"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update rocket sim spreadsheet
spreadsheet updated
</commit_message>
<xml_diff>
--- a/PROPULSION HRD-01 Diseño de banco de pruebas Maria Rev.1.xlsx
+++ b/PROPULSION HRD-01 Diseño de banco de pruebas Maria Rev.1.xlsx
@@ -1991,11 +1991,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="-1316492864"/>
-        <c:axId val="-1316504832"/>
+        <c:axId val="2081233776"/>
+        <c:axId val="2081242480"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="-1316492864"/>
+        <c:axId val="2081233776"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2052,12 +2052,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1316504832"/>
+        <c:crossAx val="2081242480"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-1316504832"/>
+        <c:axId val="2081242480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2114,7 +2114,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1316492864"/>
+        <c:crossAx val="2081233776"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2481,11 +2481,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="-1390972832"/>
-        <c:axId val="-1390973920"/>
+        <c:axId val="2081243024"/>
+        <c:axId val="2081232688"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="-1390972832"/>
+        <c:axId val="2081243024"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2542,12 +2542,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1390973920"/>
+        <c:crossAx val="2081232688"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-1390973920"/>
+        <c:axId val="2081232688"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2604,7 +2604,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1390972832"/>
+        <c:crossAx val="2081243024"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3725,11 +3725,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="-1316492320"/>
-        <c:axId val="-1316501024"/>
+        <c:axId val="2081227792"/>
+        <c:axId val="2081232144"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="-1316492320"/>
+        <c:axId val="2081227792"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3786,12 +3786,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1316501024"/>
+        <c:crossAx val="2081232144"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="-1316501024"/>
+        <c:axId val="2081232144"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="150"/>
@@ -3849,7 +3849,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-1316492320"/>
+        <c:crossAx val="2081227792"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5586,7 +5586,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5684C3C5-DAA1-0FFD-42E3-3D5DF59271BC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{5684C3C5-DAA1-0FFD-42E3-3D5DF59271BC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5635,7 +5635,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{896B3375-9C92-1B6B-758A-EA72BB08F586}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{896B3375-9C92-1B6B-758A-EA72BB08F586}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5679,7 +5679,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6CA22387-73AB-26F5-3C1D-5737F039543F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{6CA22387-73AB-26F5-3C1D-5737F039543F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5728,7 +5728,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D8E8793-F09C-DBBC-8F68-AB2AB1330A6F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{5D8E8793-F09C-DBBC-8F68-AB2AB1330A6F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5772,7 +5772,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED8B252A-7486-70B0-AC76-61C6891FB4D2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{ED8B252A-7486-70B0-AC76-61C6891FB4D2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5821,7 +5821,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7C4DA1F8-A635-4E4C-9C97-10B5703E0C0F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{7C4DA1F8-A635-4E4C-9C97-10B5703E0C0F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5882,7 +5882,7 @@
         <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{401281D1-570F-B0E7-290B-B831A7033209}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{401281D1-570F-B0E7-290B-B831A7033209}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6045,7 +6045,7 @@
         <xdr:cNvPr id="6145" name="AutoShape 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2CF56B6D-0E4C-76D3-7C78-C253C736FF53}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{2CF56B6D-0E4C-76D3-7C78-C253C736FF53}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -12279,26 +12279,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d7929c02-2ff7-4e2f-b3f4-5d7437463a37" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f5cf7016-d570-4e66-bed5-9c66354e4d60">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006416C8A108E61840AFB84A4598B73E55" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b1d8d0092a91b491fa162699921cd7b6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f5cf7016-d570-4e66-bed5-9c66354e4d60" xmlns:ns3="d7929c02-2ff7-4e2f-b3f4-5d7437463a37" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dc769dae83c42ca581dc5110a4ef7ce3" ns2:_="" ns3:_="">
     <xsd:import namespace="f5cf7016-d570-4e66-bed5-9c66354e4d60"/>
@@ -12505,26 +12485,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B672EAD0-EA6C-460E-95E6-5BDD1102E907}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d7929c02-2ff7-4e2f-b3f4-5d7437463a37"/>
-    <ds:schemaRef ds:uri="f5cf7016-d570-4e66-bed5-9c66354e4d60"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2573117B-6260-4644-A359-931F1507CA1F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d7929c02-2ff7-4e2f-b3f4-5d7437463a37" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f5cf7016-d570-4e66-bed5-9c66354e4d60">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11299929-15DA-49D6-A514-2A8A25D7CF50}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12541,4 +12522,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2573117B-6260-4644-A359-931F1507CA1F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B672EAD0-EA6C-460E-95E6-5BDD1102E907}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d7929c02-2ff7-4e2f-b3f4-5d7437463a37"/>
+    <ds:schemaRef ds:uri="f5cf7016-d570-4e66-bed5-9c66354e4d60"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>